<commit_message>
Split HubSpot Work prompt into exact build and load-rows prompts; confirm 90-day target
Prompt text is now generated from process_data.py with every task, intake
question, setup item and training module written in, so nothing has to be
pasted in by hand.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DiunCGL7n2VJA7PHAu6hWy
</commit_message>
<xml_diff>
--- a/marketing-hub-onboarding/Marketing_Hub_Onboarding_Process.xlsx
+++ b/marketing-hub-onboarding/Marketing_Hub_Onboarding_Process.xlsx
@@ -23,7 +23,7 @@
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Comms!$A$4:$E$17</definedName>
     <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'HubSpot Build Spec'!$A$4:$C$23</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Intake Form'!$A$4:$G$29</definedName>
-    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Open Questions'!$A$4:$E$15</definedName>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Open Questions'!$A$4:$E$14</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Task Template'!$A$6:$L$83</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Tech Setup'!$A$4:$F$44</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Training!$A$4:$F$13</definedName>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1534" uniqueCount="887">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="885">
   <si>
     <t xml:space="preserve">RevGravy · Marketing Hub Onboarding Process (draft v1)</t>
   </si>
@@ -2621,12 +2621,6 @@
   </si>
   <si>
     <t xml:space="preserve">Program</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is the Marketing Hub onboarding a fixed 90-day program? The roadmap assumes 90 days because of the '30 days before we finish' step.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day offsets, MBR count, 'what's next' timing</t>
   </si>
   <si>
     <t xml:space="preserve">Which Marketing Hub tiers do we sell onboarding for (Starter, Pro, Enterprise)? Is there one package or several?</t>
@@ -3523,7 +3517,7 @@
     <tabColor rgb="FF1F3A5F"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3575,18 +3569,18 @@
       </c>
       <c r="E5" s="22"/>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="E6" s="22"/>
     </row>
@@ -3595,7 +3589,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>866</v>
@@ -3610,22 +3604,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>865</v>
+        <v>868</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="E8" s="22"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>871</v>
@@ -3640,7 +3634,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>873</v>
@@ -3655,22 +3649,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="E11" s="22"/>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>878</v>
@@ -3680,12 +3674,12 @@
       </c>
       <c r="E12" s="22"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>880</v>
@@ -3695,38 +3689,23 @@
       </c>
       <c r="E13" s="22"/>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="E14" s="22"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>884</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>885</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>886</v>
-      </c>
-      <c r="E15" s="22"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:E15"/>
+  <autoFilter ref="A4:E14"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Switch the HubSpot Work design to shared tables and write one prompt per agent
HubSpot Work's build showed project copies can't carry agents or link to the
Customers table. All customers now share Customers, Customer Tasks, Requests
and Updates tables; the template's Tasks table is the master list.

- hubspot-work-redesign-prompt.txt converts the workspace already built
- hubspot-work-agent-prompts.md has 8 standalone prompts for the agent builder
- full prompt, sheet and roadmap updated to match

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DiunCGL7n2VJA7PHAu6hWy
</commit_message>
<xml_diff>
--- a/marketing-hub-onboarding/Marketing_Hub_Onboarding_Process.xlsx
+++ b/marketing-hub-onboarding/Marketing_Hub_Onboarding_Process.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="1031">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1769" uniqueCount="1043">
   <si>
     <t xml:space="preserve">RevGravy · Marketing Hub Onboarding Process (v2)</t>
   </si>
@@ -193,7 +193,7 @@
     <t xml:space="preserve">60 to 90 days.</t>
   </si>
   <si>
-    <t xml:space="preserve">The plan is laid out for 90 days. Each customer project has a Program length; later due dates compress to fit 60 or 75 days.</t>
+    <t xml:space="preserve">The plan is laid out for 90 days. Each customer has a Program length on their Customers row; later due dates compress to fit 60 or 75 days.</t>
   </si>
   <si>
     <t xml:space="preserve">Hub tiers</t>
@@ -316,10 +316,10 @@
     <t xml:space="preserve">HubSpot Work limits (found in the build)</t>
   </si>
   <si>
-    <t xml:space="preserve">No custom project fields; no links between tables and projects.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer details live on the Customers table, matched to the project by its exact name. Due date uses two helper columns that the Date Setter agent fills.</t>
+    <t xml:space="preserve">No custom project fields; copies of a project don't carry agent workflows.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All customers share one Customer Tasks, Requests and Updates table, each row linked to its Customers row. The template project's Tasks table is the master list the Task Generator copies from.</t>
   </si>
   <si>
     <t xml:space="preserve">Scope limits for migration and website work (suggested)</t>
@@ -454,7 +454,7 @@
     <t xml:space="preserve">Welcome email series with the Supered Action Plan (expectations, next steps, links, agreement, to-dos).</t>
   </si>
   <si>
-    <t xml:space="preserve">Architect assigned, Phil↔Architect 1:1 done, customer project created, kickoff booked.</t>
+    <t xml:space="preserve">Architect assigned, Phil↔Architect 1:1 done, customer added in HubSpot Work with tasks created, kickoff booked.</t>
   </si>
   <si>
     <t xml:space="preserve">P2</t>
@@ -766,13 +766,13 @@
     <t xml:space="preserve">1.02</t>
   </si>
   <si>
-    <t xml:space="preserve">Create the customer project</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duplicate the 'Marketing Hub Onboarding (Template)' project and name it exactly '&lt;Client&gt; · Marketing Hub Onboarding'. Add a Customers row with that exact name plus Company, Deal, Architect, Program length and Start date. Share the project with the Architect.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work: customer project + Customers row</t>
+    <t xml:space="preserve">Add the customer in HubSpot Work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add a Customers row: Customer, Company, Deal, Architect, Program length, Start date, tier, From→To goal, FigJam and Supered links. Check that the Task Generator created the customer's tasks (Tasks created = Yes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work: Customers table</t>
   </si>
   <si>
     <t xml:space="preserve">1.03</t>
@@ -817,10 +817,10 @@
     <t xml:space="preserve">Set up progress measures</t>
   </si>
   <si>
-    <t xml:space="preserve">Add the customer's progress measures to the project (name '&lt;Client&gt; 1.1 Visitor to Lead' etc.) with baseline, target and schedule.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work: customer project</t>
+    <t xml:space="preserve">Add the customer's progress measures to their Customers row (name '&lt;Client&gt; 1.1 Visitor to Lead' etc.) with baseline, target and schedule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work: Customers row</t>
   </si>
   <si>
     <t xml:space="preserve">1.07</t>
@@ -925,7 +925,7 @@
     <t xml:space="preserve">Data health, email health, existing assets, tracking, workflows, properties, old tool inventory. 1-page summary for kickoff.</t>
   </si>
   <si>
-    <t xml:space="preserve">Work: customer project (notes)</t>
+    <t xml:space="preserve">Work: Updates table</t>
   </si>
   <si>
     <t xml:space="preserve">2.07</t>
@@ -2632,7 +2632,7 @@
     <t xml:space="preserve">HubSpot Work</t>
   </si>
   <si>
-    <t xml:space="preserve">The whole onboarding: a template project copied per customer (tasks by section, board, timeline, requests) and a Customers table where each customer's details live.</t>
+    <t xml:space="preserve">The whole onboarding: one shared set of tables for all customers (Customers, Customer Tasks, Requests, Updates), a template task list, board, timeline and agents.</t>
   </si>
   <si>
     <t xml:space="preserve">Everything the customer sees: Action Plan, announcements, delivery and training videos, admin handbook.</t>
@@ -2650,7 +2650,7 @@
     <t xml:space="preserve">Projects object pipelines, tickets, HubSpot customer portal, Trello.</t>
   </si>
   <si>
-    <t xml:space="preserve">Setting up a new customer (HubSpot Work has no custom project fields)</t>
+    <t xml:space="preserve">Setting up a new customer (all customers share the same tables)</t>
   </si>
   <si>
     <t xml:space="preserve">Step</t>
@@ -2659,19 +2659,19 @@
     <t xml:space="preserve">What to do</t>
   </si>
   <si>
-    <t xml:space="preserve">Duplicate 'Marketing Hub Onboarding (Template)' and name the copy exactly '&lt;Client&gt; · Marketing Hub Onboarding'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add a row to Customers with Customer = that exact name, plus Company, Deal, Architect, Program length, Start date and the rest.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Date Setter agent fills Project Day 0 and Program length on every task in the copy, so Due dates calculate. Without the agent, bulk-edit those two columns on all rows.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Share the copy with the Architect (workspaces are private by default).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Template project 'Marketing Hub Onboarding (Template)': Tasks table columns</t>
+    <t xml:space="preserve">Add a row to Customers: Customer, Company, Deal, Architect, Program length, Start date, tier, From→To goal, FigJam and Supered links.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Task Generator agent copies the template tasks into Customer Tasks for that customer, fills the dates, assigns the Architect and sets Tasks created = Yes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To work on one customer, filter any view by Customer. 'My tasks' shows an Architect's work across all their customers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share the workspace with Phil and the Architects (it's private by default).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task columns (template Tasks table and the shared Customer Tasks table, which adds a Customer link)</t>
   </si>
   <si>
     <t xml:space="preserve">Column</t>
@@ -2767,10 +2767,10 @@
     <t xml:space="preserve">Project Day 0</t>
   </si>
   <si>
-    <t xml:space="preserve">Helper for the formula: same date on every row, filled per customer (hidden)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Helper for the formula: 60, 75 or 90 on every row, filled per customer (hidden)</t>
+    <t xml:space="preserve">Helper for the formula: the customer's Start date, filled by the Task Generator (hidden)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helper for the formula: 60, 75 or 90, filled by the Task Generator (hidden)</t>
   </si>
   <si>
     <t xml:space="preserve">Board statuses</t>
@@ -2806,7 +2806,13 @@
     <t xml:space="preserve">Board</t>
   </si>
   <si>
-    <t xml:space="preserve">Columns = Status. Cards show Task ID, Task, Assignee, Due date.</t>
+    <t xml:space="preserve">Columns = Status. Cards show Customer, Task ID, Task, Assignee, Due date.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List grouped by Customer, then Section, sorted by Task ID.</t>
   </si>
   <si>
     <t xml:space="preserve">By section</t>
@@ -2818,7 +2824,7 @@
     <t xml:space="preserve">Timeline</t>
   </si>
   <si>
-    <t xml:space="preserve">Start date → Due date, grouped by Section.</t>
+    <t xml:space="preserve">Start date → Due date, grouped by Customer.</t>
   </si>
   <si>
     <t xml:space="preserve">Calendar</t>
@@ -2851,7 +2857,13 @@
     <t xml:space="preserve">Due date before today, Status not Done / Won't do.</t>
   </si>
   <si>
-    <t xml:space="preserve">Requests table (one per customer project)</t>
+    <t xml:space="preserve">Requests table (shared, each row linked to its customer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link to Customers row</t>
   </si>
   <si>
     <t xml:space="preserve">Request</t>
@@ -2866,19 +2878,34 @@
     <t xml:space="preserve">Dropdown: New, Quoted, In progress, Done, Parked</t>
   </si>
   <si>
-    <t xml:space="preserve">Number (default 250)</t>
+    <t xml:space="preserve">Number, default 250</t>
   </si>
   <si>
     <t xml:space="preserve">Logged on</t>
   </si>
   <si>
-    <t xml:space="preserve">Portfolio project 'Onboarding Portfolio': Customers table, one row per customer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Text: the customer project's exact name, '&lt;Client&gt; · Marketing Hub Onboarding'</t>
+    <t xml:space="preserve">Updates table (drafts the agents write for the Architect)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dropdown: Handoff brief, Weekly update, What's next options, KPI snapshot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date: week of, or month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dropdown: Draft, Reviewed, Sent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers table, one row per customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text: client name</t>
   </si>
   <si>
     <t xml:space="preserve">Company</t>
@@ -2893,7 +2920,7 @@
     <t xml:space="preserve">Number: 60, 75 or 90</t>
   </si>
   <si>
-    <t xml:space="preserve">Date (Day 0)</t>
+    <t xml:space="preserve">Date, Day 0</t>
   </si>
   <si>
     <t xml:space="preserve">Target end date</t>
@@ -2917,12 +2944,21 @@
     <t xml:space="preserve">Next MBR</t>
   </si>
   <si>
+    <t xml:space="preserve">Date, filled by the Architect when booked</t>
+  </si>
+  <si>
     <t xml:space="preserve">Next due task</t>
   </si>
   <si>
+    <t xml:space="preserve">Tasks created</t>
+  </si>
+  <si>
     <t xml:space="preserve">From→To goal</t>
   </si>
   <si>
+    <t xml:space="preserve">Long text: name, baseline, target</t>
+  </si>
+  <si>
     <t xml:space="preserve">FigJam link</t>
   </si>
   <si>
@@ -2938,7 +2974,7 @@
     <t xml:space="preserve">Capacity</t>
   </si>
   <si>
-    <t xml:space="preserve">Report: active customers per Architect (a report, since saved views can't count). Phil uses it to pick the Architect.</t>
+    <t xml:space="preserve">Report: active customers per Architect. Phil uses it to pick the Architect.</t>
   </si>
   <si>
     <t xml:space="preserve">Health board</t>
@@ -2953,7 +2989,7 @@
     <t xml:space="preserve">Target end date in the next 35 days (time for the 'what's next' call).</t>
   </si>
   <si>
-    <t xml:space="preserve">Agents (draft, fill dates or flag only; none sends anything to a customer)</t>
+    <t xml:space="preserve">Agents (draft, fill fields or flag only; none sends anything to a customer). Full prompts: hubspot-work-agent-prompts.md</t>
   </si>
   <si>
     <t xml:space="preserve">Agent</t>
@@ -2965,76 +3001,76 @@
     <t xml:space="preserve">What it does</t>
   </si>
   <si>
-    <t xml:space="preserve">Date Setter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Customers row's Start date, Program length or Architect is set or changed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Find the project whose name matches the row's Customer value. In its Tasks table, set Project Day 0 = the row's Start date and Program length = the row's Program length on every task, so the Due date formula calculates. Assign every task with Owner role 'Architect' to the row's Architect. Set the row's Target end date = Start date + Program length.</t>
+    <t xml:space="preserve">Onboarding Task Generator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A row in the Customers table has Start date, Program length and Architect filled, and Tasks created is not Yes. Also run when Start date, Program length or Architect changes on a row where Tasks created is Yes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copies the template tasks into Customer Tasks for a new customer, fills the dates and assigns the Architect.</t>
   </si>
   <si>
     <t xml:space="preserve">Handoff Brief</t>
   </si>
   <si>
-    <t xml:space="preserve">A new row in Customers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read the linked deal's history, notes, meetings and emails. Write a one-page brief for the Architect: who the customer is, the From→To goal, what they bought, the progress measures, the people involved, risks and open questions. Save it in the matching customer project and notify the Architect.</t>
+    <t xml:space="preserve">Tasks created changes to Yes on a Customers row.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Writes a one-page brief for the Architect from the deal's history.</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly Update Drafter</t>
   </si>
   <si>
-    <t xml:space="preserve">Every Thursday, for each Customers row whose Current section is P2 to P8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In the matching project, draft the Friday update in five parts: 1) work done this week and the strategic issue it moves, 2) numbers vs baseline, 3) issues found outside scope, 4) next week, 5) client to-dos. Use tasks marked Done this week, tasks due next week, and Requests logged this week. Save the draft in the project and notify the Architect, who reviews and sends it.</t>
+    <t xml:space="preserve">Every Thursday at 9:00 AM (America/Phoenix).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drafts each customer's Friday update for the Architect to review and send.</t>
   </si>
   <si>
     <t xml:space="preserve">Delay Flagger</t>
   </si>
   <si>
-    <t xml:space="preserve">Every weekday morning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In each customer project, flag tasks past their Due date and tasks 'Waiting on client' for more than 3 days. If a project has 3 or more overdue tasks, set Health to At risk on its Customers row. Notify the Architect, and notify Phil when Health becomes At risk or Off track.</t>
+    <t xml:space="preserve">Every weekday at 8:00 AM (America/Phoenix).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flags overdue and stuck tasks and sets Health to At risk.</t>
   </si>
   <si>
     <t xml:space="preserve">Request Triage</t>
   </si>
   <si>
-    <t xml:space="preserve">A new row in a customer project's Requests table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suggest the Urgency class and Price from the urgency rules, and set Due date from that class's turnaround. If it looks bigger than about 2 hours of work, mark it 'Quoted' and say why. Notify the Architect at once for Critical requests.</t>
+    <t xml:space="preserve">A new row is added to the Requests table.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suggests the urgency class, price and due date for each new request.</t>
   </si>
   <si>
     <t xml:space="preserve">Portfolio Sync</t>
   </si>
   <si>
-    <t xml:space="preserve">Every day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For each Customers row, look at the matching project and update Current section (earliest section with open tasks), Next MBR and Next due task.</t>
+    <t xml:space="preserve">Every day at 6:00 AM (America/Phoenix).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keeps each customer's Current section and Next due task up to date.</t>
   </si>
   <si>
     <t xml:space="preserve">What's Next Prep</t>
   </si>
   <si>
-    <t xml:space="preserve">35 days before a Customers row's Target end date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summarize results vs baseline, issues found and 'not now' requests into Option A and Option B for the next phase. Save it in the matching project, notify the Architect, and ask Phil to review before the call.</t>
+    <t xml:space="preserve">Every day at 7:00 AM (America/Phoenix), for Customers rows whose Target end date is 35 days away or less and that don't have a 'What's next options' update yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepares Option A and Option B for the 'what's next' call.</t>
   </si>
   <si>
     <t xml:space="preserve">KPI Snapshot Drafter</t>
   </si>
   <si>
-    <t xml:space="preserve">Monthly for 6 months after a Customers row's Target end date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft the monthly KPI snapshot notes (3 short notes on the progress measures) for the Architect to review and send with the dashboard email.</t>
+    <t xml:space="preserve">The 1st of every month at 9:00 AM (America/Phoenix).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drafts the monthly KPI notes during the 6 months of free monitoring.</t>
   </si>
   <si>
     <t xml:space="preserve">Tool Fit: HubSpot Work vs Projects vs Tickets</t>
@@ -4452,7 +4488,7 @@
     <tabColor rgb="FF2E7D7A"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="26"/>
@@ -4551,7 +4587,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
         <v>3</v>
       </c>
@@ -4912,379 +4948,483 @@
         <v>935</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="s">
         <v>936</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3" t="s">
+      <c r="B57" s="4"/>
+      <c r="C57" s="4" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="5" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
         <v>877</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B60" s="3" t="s">
         <v>878</v>
       </c>
-      <c r="C59" s="3"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
-        <v>937</v>
-      </c>
-      <c r="B60" s="4" t="s">
+      <c r="C60" s="3"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4" t="s">
+        <v>939</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>940</v>
+      </c>
+      <c r="C61" s="4"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="s">
+        <v>941</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>578</v>
-      </c>
-      <c r="C60" s="4"/>
-    </row>
-    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="s">
-        <v>536</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>938</v>
-      </c>
-      <c r="C61" s="4"/>
-    </row>
-    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="s">
-        <v>878</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>939</v>
       </c>
       <c r="C62" s="4"/>
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>942</v>
+      </c>
+      <c r="C63" s="4"/>
+    </row>
+    <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>878</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>943</v>
+      </c>
+      <c r="C64" s="4"/>
+    </row>
+    <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
         <v>882</v>
       </c>
-      <c r="B63" s="4" t="s">
-        <v>940</v>
-      </c>
-      <c r="C63" s="4"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="4" t="s">
-        <v>539</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>941</v>
-      </c>
-      <c r="C64" s="4"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="4" t="s">
-        <v>942</v>
-      </c>
       <c r="B65" s="4" t="s">
-        <v>905</v>
+        <v>944</v>
       </c>
       <c r="C65" s="4"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>890</v>
+        <v>539</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>905</v>
+        <v>945</v>
       </c>
       <c r="C66" s="4"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
+        <v>946</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>905</v>
+      </c>
+      <c r="C67" s="4"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>890</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>905</v>
+      </c>
+      <c r="C68" s="4"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
         <v>879</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B69" s="4" t="s">
         <v>897</v>
       </c>
-      <c r="C67" s="4"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="s">
-        <v>943</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="3" t="s">
+      <c r="C69" s="4"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
         <v>877</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="B72" s="3" t="s">
         <v>878</v>
       </c>
-      <c r="C70" s="3"/>
-    </row>
-    <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="4" t="s">
-        <v>944</v>
-      </c>
-      <c r="B71" s="4" t="s">
-        <v>945</v>
-      </c>
-      <c r="C71" s="4"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="4" t="s">
-        <v>946</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>947</v>
-      </c>
-      <c r="C72" s="4"/>
+      <c r="C72" s="3"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
-        <v>464</v>
+        <v>939</v>
       </c>
       <c r="B73" s="4" t="s">
+        <v>940</v>
+      </c>
+      <c r="C73" s="4"/>
+    </row>
+    <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="4" t="s">
+        <v>878</v>
+      </c>
+      <c r="B74" s="4" t="s">
         <v>948</v>
-      </c>
-      <c r="C73" s="4"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B74" s="4" t="s">
-        <v>888</v>
       </c>
       <c r="C74" s="4"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="s">
-        <v>48</v>
+        <v>949</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="C75" s="4"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="s">
-        <v>904</v>
+        <v>951</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>950</v>
+        <v>897</v>
       </c>
       <c r="C76" s="4"/>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>951</v>
+        <v>882</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>905</v>
+        <v>952</v>
       </c>
       <c r="C77" s="4"/>
     </row>
-    <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="s">
-        <v>625</v>
+        <v>879</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>952</v>
+        <v>897</v>
       </c>
       <c r="C78" s="4"/>
     </row>
-    <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="4" t="s">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="5" t="s">
         <v>953</v>
       </c>
-      <c r="B79" s="4" t="s">
-        <v>954</v>
-      </c>
-      <c r="C79" s="4"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="4" t="s">
-        <v>955</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>956</v>
-      </c>
-      <c r="C80" s="4"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="4" t="s">
-        <v>957</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>905</v>
-      </c>
-      <c r="C81" s="4"/>
+    </row>
+    <row r="81" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="C81" s="3"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="s">
-        <v>958</v>
+        <v>939</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>578</v>
+        <v>954</v>
       </c>
       <c r="C82" s="4"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>897</v>
+        <v>956</v>
       </c>
       <c r="C83" s="4"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="s">
-        <v>960</v>
+        <v>464</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="C84" s="4"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>888</v>
+      </c>
+      <c r="C85" s="4"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>958</v>
+      </c>
+      <c r="C86" s="4"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="4" t="s">
+        <v>904</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>959</v>
+      </c>
+      <c r="C87" s="4"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="4" t="s">
+        <v>960</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>905</v>
+      </c>
+      <c r="C88" s="4"/>
+    </row>
+    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="4" t="s">
+        <v>625</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>961</v>
+      </c>
+      <c r="C89" s="4"/>
+    </row>
+    <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="4" t="s">
         <v>962</v>
       </c>
-      <c r="B85" s="4" t="s">
-        <v>961</v>
-      </c>
-      <c r="C85" s="4"/>
-    </row>
-    <row r="87" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="3" t="s">
+      <c r="B90" s="4" t="s">
         <v>963</v>
       </c>
-      <c r="B87" s="3"/>
-      <c r="C87" s="3" t="s">
+      <c r="C90" s="4"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="4" t="s">
+        <v>964</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>965</v>
+      </c>
+      <c r="C91" s="4"/>
+    </row>
+    <row r="92" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="4" t="s">
+        <v>966</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>967</v>
+      </c>
+      <c r="C92" s="4"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="4" t="s">
+        <v>968</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="C93" s="4"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="4" t="s">
+        <v>969</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="C94" s="4"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="4" t="s">
+        <v>970</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>897</v>
+      </c>
+      <c r="C95" s="4"/>
+    </row>
+    <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>971</v>
+      </c>
+      <c r="C96" s="4"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="4" t="s">
+        <v>972</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>973</v>
+      </c>
+      <c r="C97" s="4"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="4" t="s">
+        <v>974</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>973</v>
+      </c>
+      <c r="C98" s="4"/>
+    </row>
+    <row r="100" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="3" t="s">
+        <v>975</v>
+      </c>
+      <c r="B100" s="3"/>
+      <c r="C100" s="3" t="s">
         <v>919</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="4" t="s">
-        <v>964</v>
-      </c>
-      <c r="B88" s="4"/>
-      <c r="C88" s="4" t="s">
-        <v>965</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="4" t="s">
-        <v>966</v>
-      </c>
-      <c r="B89" s="4"/>
-      <c r="C89" s="4" t="s">
-        <v>967</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="4" t="s">
-        <v>968</v>
-      </c>
-      <c r="B90" s="4"/>
-      <c r="C90" s="4" t="s">
-        <v>969</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="5" t="s">
-        <v>970</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="8" t="s">
-        <v>971</v>
-      </c>
-      <c r="B93" s="8" t="s">
-        <v>972</v>
-      </c>
-      <c r="C93" s="8" t="s">
-        <v>973</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="4" t="s">
-        <v>974</v>
-      </c>
-      <c r="B94" s="4" t="s">
-        <v>975</v>
-      </c>
-      <c r="C94" s="4" t="s">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="4" t="s">
         <v>976</v>
       </c>
-    </row>
-    <row r="95" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="4" t="s">
+      <c r="B101" s="4"/>
+      <c r="C101" s="4" t="s">
         <v>977</v>
       </c>
-      <c r="B95" s="4" t="s">
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="4" t="s">
         <v>978</v>
       </c>
-      <c r="C95" s="4" t="s">
+      <c r="B102" s="4"/>
+      <c r="C102" s="4" t="s">
         <v>979</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="4" t="s">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="4" t="s">
         <v>980</v>
       </c>
-      <c r="B96" s="4" t="s">
+      <c r="B103" s="4"/>
+      <c r="C103" s="4" t="s">
         <v>981</v>
       </c>
-      <c r="C96" s="4" t="s">
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="5" t="s">
         <v>982</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="4" t="s">
+    <row r="106" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="8" t="s">
         <v>983</v>
       </c>
-      <c r="B97" s="4" t="s">
+      <c r="B106" s="8" t="s">
         <v>984</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C106" s="8" t="s">
         <v>985</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="4" t="s">
+    <row r="107" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="4" t="s">
         <v>986</v>
       </c>
-      <c r="B98" s="4" t="s">
+      <c r="B107" s="4" t="s">
         <v>987</v>
       </c>
-      <c r="C98" s="4" t="s">
+      <c r="C107" s="4" t="s">
         <v>988</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="4" t="s">
+    <row r="108" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="4" t="s">
         <v>989</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B108" s="4" t="s">
         <v>990</v>
       </c>
-      <c r="C99" s="4" t="s">
+      <c r="C108" s="4" t="s">
         <v>991</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="4" t="s">
+    <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="4" t="s">
         <v>992</v>
       </c>
-      <c r="B100" s="4" t="s">
+      <c r="B109" s="4" t="s">
         <v>993</v>
       </c>
-      <c r="C100" s="4" t="s">
+      <c r="C109" s="4" t="s">
         <v>994</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="4" t="s">
+    <row r="110" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="4" t="s">
         <v>995</v>
       </c>
-      <c r="B101" s="4" t="s">
+      <c r="B110" s="4" t="s">
         <v>996</v>
       </c>
-      <c r="C101" s="4" t="s">
+      <c r="C110" s="4" t="s">
         <v>997</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="4" t="s">
+        <v>998</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>999</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="4" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="4" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="4" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>1009</v>
       </c>
     </row>
   </sheetData>
@@ -5318,201 +5458,201 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>998</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>999</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>1000</v>
+        <v>1012</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1001</v>
+        <v>1013</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>862</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>1002</v>
+        <v>1014</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>1003</v>
+        <v>1015</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>1004</v>
+        <v>1016</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>1004</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>1005</v>
+        <v>1017</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>1006</v>
+        <v>1018</v>
       </c>
       <c r="D5" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>1007</v>
+        <v>1019</v>
       </c>
       <c r="F5" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>1008</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>1009</v>
+        <v>1021</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>1010</v>
+        <v>1022</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>1011</v>
+        <v>1023</v>
       </c>
       <c r="F6" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>1012</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>1013</v>
+        <v>1025</v>
       </c>
       <c r="B7" s="15" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>1014</v>
+        <v>1026</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>1015</v>
+        <v>1027</v>
       </c>
       <c r="F7" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>1016</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>1017</v>
+        <v>1029</v>
       </c>
       <c r="B8" s="15" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>1018</v>
+        <v>1030</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>1019</v>
+        <v>1031</v>
       </c>
       <c r="F8" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>1019</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>1020</v>
+        <v>1032</v>
       </c>
       <c r="B9" s="15" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>1021</v>
+        <v>1033</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>1022</v>
+        <v>1034</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>1022</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>1023</v>
+        <v>1035</v>
       </c>
       <c r="B10" s="15" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>1024</v>
+        <v>1036</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>1025</v>
+        <v>1037</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>1026</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>1027</v>
+        <v>1039</v>
       </c>
       <c r="B11" s="15" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>1028</v>
+        <v>1040</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
       <c r="F11" s="15" t="n">
         <v>2</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>1030</v>
+        <v>1042</v>
       </c>
       <c r="B12" s="20" t="n">
         <f aca="false">SUM(B5:B11)</f>
@@ -5776,7 +5916,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
@@ -8021,7 +8161,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>240</v>
       </c>

</xml_diff>